<commit_message>
document register logic fixed, still need to fix project_id logic and parse error
</commit_message>
<xml_diff>
--- a/docs/GE2ExcelTestFile.xlsx
+++ b/docs/GE2ExcelTestFile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryanmichaelnuera/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D2458DE-DF1A-BD46-98EC-21649627E189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDA16F44-1CB8-C44C-9D38-51A5142A189B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GE2 2026 F1 ECBV" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="555">
   <si>
     <t>VARIABLE</t>
   </si>
@@ -1741,13 +1741,22 @@
     <t>Input file not found.</t>
   </si>
   <si>
-    <t>994da7c4d18c65f0dfc5715848fe132556d0f80e705a0e8d620c79939de29e31</t>
-  </si>
-  <si>
-    <t>0abec6611f29374af22889bec468e450657aaa9832886a449fe2d4f937d23295</t>
-  </si>
-  <si>
-    <t>1339927c516401a3dfe3ca7720347c9a4db73f4a20c086ecd315446e6483575e</t>
+    <t>fe2db16b6daf5aefa4b28a411c457632c64264297c59c51017dcc7a4d3996619</t>
+  </si>
+  <si>
+    <t>8a928247c536e01c50724ece39830fe4bbceb25c1923fcf9e2fcc7a5c064822d</t>
+  </si>
+  <si>
+    <t>43581708ae9e6dbe6e50d97e99fb04e3d87c92571d501237b4ffbb96d556dcca</t>
+  </si>
+  <si>
+    <t>This file is not JSON formatted.</t>
+  </si>
+  <si>
+    <t>JSON does not have the expected structure.</t>
+  </si>
+  <si>
+    <t>JSON data has no valid values.</t>
   </si>
 </sst>
 </file>
@@ -2131,7 +2140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2291,9 +2300,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -8080,7 +8086,7 @@
     <col min="6" max="6" width="28.7109375" customWidth="1"/>
     <col min="7" max="7" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="59" customWidth="1"/>
-    <col min="9" max="9" width="57.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="60.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="14" width="10.42578125" customWidth="1"/>
     <col min="15" max="15" width="11.42578125" bestFit="1" customWidth="1"/>
@@ -8289,7 +8295,7 @@
         <v>547</v>
       </c>
       <c r="I6" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J6" s="62"/>
       <c r="O6" s="47"/>
@@ -8320,7 +8326,7 @@
         <v>480</v>
       </c>
       <c r="I7" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J7" s="62"/>
       <c r="O7" s="47"/>
@@ -8351,7 +8357,7 @@
         <v>481</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J8" s="62"/>
     </row>
@@ -8381,7 +8387,7 @@
         <v>482</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J9" s="62"/>
     </row>
@@ -8411,7 +8417,7 @@
         <v>265</v>
       </c>
       <c r="I10" s="30" t="s">
-        <v>140</v>
+        <v>553</v>
       </c>
       <c r="J10" s="62"/>
     </row>
@@ -8441,7 +8447,7 @@
         <v>544</v>
       </c>
       <c r="I11" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J11" s="62"/>
     </row>
@@ -8471,7 +8477,7 @@
         <v>475</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J12" s="62"/>
     </row>
@@ -8501,7 +8507,7 @@
         <v>476</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J13" s="62"/>
     </row>
@@ -8531,7 +8537,7 @@
         <v>483</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J14" s="62"/>
     </row>
@@ -8557,11 +8563,11 @@
       <c r="G15" s="65" t="s">
         <v>281</v>
       </c>
-      <c r="H15" s="70" t="s">
+      <c r="H15" s="69" t="s">
         <v>484</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J15" s="62"/>
     </row>
@@ -8591,7 +8597,7 @@
         <v>543</v>
       </c>
       <c r="I16" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J16" s="62"/>
     </row>
@@ -8621,7 +8627,7 @@
         <v>485</v>
       </c>
       <c r="I17" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J17" s="62"/>
     </row>
@@ -8651,7 +8657,7 @@
         <v>486</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J18" s="62"/>
     </row>
@@ -8681,7 +8687,7 @@
         <v>487</v>
       </c>
       <c r="I19" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J19" s="62"/>
     </row>
@@ -8711,7 +8717,7 @@
         <v>490</v>
       </c>
       <c r="I20" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J20" s="62"/>
     </row>
@@ -8741,7 +8747,7 @@
         <v>545</v>
       </c>
       <c r="I21" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J21" s="62"/>
     </row>
@@ -8771,7 +8777,7 @@
         <v>496</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J22" s="62"/>
     </row>
@@ -8801,7 +8807,7 @@
         <v>500</v>
       </c>
       <c r="I23" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J23" s="62"/>
     </row>
@@ -8831,7 +8837,7 @@
         <v>510</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J24" s="62"/>
     </row>
@@ -8861,7 +8867,7 @@
         <v>513</v>
       </c>
       <c r="I25" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J25" s="62"/>
     </row>
@@ -8891,7 +8897,7 @@
         <v>516</v>
       </c>
       <c r="I26" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J26" s="62"/>
     </row>
@@ -8921,7 +8927,7 @@
         <v>520</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J27" s="62"/>
     </row>
@@ -8951,7 +8957,7 @@
         <v>521</v>
       </c>
       <c r="I28" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J28" s="62"/>
     </row>
@@ -8981,7 +8987,7 @@
         <v>522</v>
       </c>
       <c r="I29" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J29" s="62"/>
     </row>
@@ -9011,7 +9017,7 @@
         <v>523</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J30" s="62"/>
     </row>
@@ -9041,7 +9047,7 @@
         <v>525</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J31" s="62"/>
     </row>
@@ -9071,7 +9077,7 @@
         <v>527</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J32" s="62"/>
     </row>
@@ -9101,7 +9107,7 @@
         <v>529</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J33" s="62"/>
     </row>
@@ -9131,7 +9137,7 @@
         <v>532</v>
       </c>
       <c r="I34" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J34" s="62"/>
     </row>
@@ -9161,7 +9167,7 @@
         <v>540</v>
       </c>
       <c r="I35" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J35" s="62"/>
     </row>
@@ -9191,7 +9197,7 @@
         <v>539</v>
       </c>
       <c r="I36" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J36" s="62"/>
     </row>
@@ -9221,7 +9227,7 @@
         <v>538</v>
       </c>
       <c r="I37" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J37" s="62"/>
     </row>
@@ -9251,7 +9257,7 @@
         <v>537</v>
       </c>
       <c r="I38" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J38" s="62"/>
     </row>
@@ -9281,7 +9287,7 @@
         <v>536</v>
       </c>
       <c r="I39" s="30" t="s">
-        <v>140</v>
+        <v>553</v>
       </c>
       <c r="J39" s="62"/>
     </row>
@@ -9311,7 +9317,7 @@
         <v>535</v>
       </c>
       <c r="I40" s="30" t="s">
-        <v>140</v>
+        <v>553</v>
       </c>
       <c r="J40" s="62"/>
     </row>
@@ -9341,7 +9347,7 @@
         <v>534</v>
       </c>
       <c r="I41" s="30" t="s">
-        <v>140</v>
+        <v>553</v>
       </c>
       <c r="J41" s="62"/>
     </row>
@@ -9371,7 +9377,7 @@
         <v>533</v>
       </c>
       <c r="I42" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J42" s="62"/>
     </row>
@@ -9401,7 +9407,7 @@
         <v>531</v>
       </c>
       <c r="I43" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J43" s="62"/>
     </row>
@@ -9431,7 +9437,7 @@
         <v>530</v>
       </c>
       <c r="I44" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J44" s="62"/>
     </row>
@@ -9461,7 +9467,7 @@
         <v>541</v>
       </c>
       <c r="I45" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J45" s="62"/>
     </row>
@@ -9491,7 +9497,7 @@
         <v>528</v>
       </c>
       <c r="I46" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J46" s="62"/>
     </row>
@@ -9521,7 +9527,7 @@
         <v>526</v>
       </c>
       <c r="I47" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J47" s="62"/>
     </row>
@@ -9551,7 +9557,7 @@
         <v>546</v>
       </c>
       <c r="I48" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J48" s="62"/>
     </row>
@@ -9581,7 +9587,7 @@
         <v>524</v>
       </c>
       <c r="I49" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J49" s="62"/>
     </row>
@@ -9611,7 +9617,7 @@
         <v>542</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J50" s="62"/>
     </row>
@@ -9641,7 +9647,7 @@
         <v>519</v>
       </c>
       <c r="I51" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J51" s="62"/>
     </row>
@@ -9671,7 +9677,7 @@
         <v>518</v>
       </c>
       <c r="I52" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J52" s="62"/>
     </row>
@@ -9701,7 +9707,7 @@
         <v>517</v>
       </c>
       <c r="I53" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J53" s="62"/>
     </row>
@@ -9731,7 +9737,7 @@
         <v>515</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J54" s="62"/>
     </row>
@@ -9761,7 +9767,7 @@
         <v>514</v>
       </c>
       <c r="I55" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J55" s="62"/>
     </row>
@@ -9791,7 +9797,7 @@
         <v>512</v>
       </c>
       <c r="I56" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J56" s="62"/>
     </row>
@@ -9821,7 +9827,7 @@
         <v>511</v>
       </c>
       <c r="I57" s="30" t="s">
-        <v>140</v>
+        <v>553</v>
       </c>
       <c r="J57" s="62"/>
     </row>
@@ -9851,7 +9857,7 @@
         <v>509</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>140</v>
+        <v>553</v>
       </c>
       <c r="J58" s="62"/>
     </row>
@@ -9881,7 +9887,7 @@
         <v>508</v>
       </c>
       <c r="I59" s="30" t="s">
-        <v>140</v>
+        <v>553</v>
       </c>
       <c r="J59" s="62"/>
     </row>
@@ -9911,7 +9917,7 @@
         <v>507</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J60" s="62"/>
     </row>
@@ -9941,7 +9947,7 @@
         <v>506</v>
       </c>
       <c r="I61" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J61" s="62"/>
     </row>
@@ -9971,7 +9977,7 @@
         <v>505</v>
       </c>
       <c r="I62" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J62" s="62"/>
     </row>
@@ -10001,7 +10007,7 @@
         <v>504</v>
       </c>
       <c r="I63" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J63" s="62"/>
     </row>
@@ -10031,7 +10037,7 @@
         <v>503</v>
       </c>
       <c r="I64" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J64" s="62"/>
     </row>
@@ -10061,7 +10067,7 @@
         <v>502</v>
       </c>
       <c r="I65" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J65" s="62"/>
     </row>
@@ -10091,7 +10097,7 @@
         <v>501</v>
       </c>
       <c r="I66" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J66" s="62"/>
     </row>
@@ -10121,7 +10127,7 @@
         <v>499</v>
       </c>
       <c r="I67" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J67" s="62"/>
     </row>
@@ -10151,7 +10157,7 @@
         <v>498</v>
       </c>
       <c r="I68" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J68" s="62"/>
     </row>
@@ -10181,7 +10187,7 @@
         <v>497</v>
       </c>
       <c r="I69" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J69" s="62"/>
     </row>
@@ -10211,7 +10217,7 @@
         <v>495</v>
       </c>
       <c r="I70" s="30" t="s">
-        <v>140</v>
+        <v>552</v>
       </c>
       <c r="J70" s="62"/>
     </row>
@@ -10219,7 +10225,7 @@
       <c r="A71" s="63">
         <v>70</v>
       </c>
-      <c r="B71" s="70" t="s">
+      <c r="B71" s="69" t="s">
         <v>448</v>
       </c>
       <c r="C71" s="51" t="s">
@@ -10241,7 +10247,7 @@
         <v>494</v>
       </c>
       <c r="I71" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J71" s="62"/>
     </row>
@@ -10249,7 +10255,7 @@
       <c r="A72" s="63">
         <v>71</v>
       </c>
-      <c r="B72" s="70" t="s">
+      <c r="B72" s="69" t="s">
         <v>448</v>
       </c>
       <c r="C72" s="51" t="s">
@@ -10271,7 +10277,7 @@
         <v>493</v>
       </c>
       <c r="I72" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J72" s="62"/>
     </row>
@@ -10279,7 +10285,7 @@
       <c r="A73" s="63">
         <v>72</v>
       </c>
-      <c r="B73" s="70">
+      <c r="B73" s="69">
         <v>49</v>
       </c>
       <c r="C73" s="51" t="s">
@@ -10301,7 +10307,7 @@
         <v>492</v>
       </c>
       <c r="I73" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J73" s="62"/>
     </row>
@@ -10331,7 +10337,7 @@
         <v>491</v>
       </c>
       <c r="I74" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J74" s="62"/>
     </row>
@@ -10361,7 +10367,7 @@
         <v>489</v>
       </c>
       <c r="I75" s="30" t="s">
-        <v>140</v>
+        <v>554</v>
       </c>
       <c r="J75" s="62"/>
     </row>
@@ -10387,13 +10393,13 @@
       <c r="G76" s="58" t="s">
         <v>466</v>
       </c>
-      <c r="H76" s="71" t="s">
+      <c r="H76" s="70" t="s">
         <v>488</v>
       </c>
-      <c r="I76" s="68" t="s">
-        <v>140</v>
-      </c>
-      <c r="J76" s="69"/>
+      <c r="I76" s="30" t="s">
+        <v>554</v>
+      </c>
+      <c r="J76" s="68"/>
     </row>
     <row r="77" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F77" s="52"/>

</xml_diff>